<commit_message>
Mobile sem overflow, data de atualização no mapa, textos corrigidos
- mapa.css: abaixo de 480px o título esconde e o nav encolhe mais (padding,
  fonte e as setinhas ▾ somem) -- "Pendências" ficava cortado fora da tela
  em celular, sem como clicar. Testado em 375px: sem overflow horizontal.
- Sidebar mostra "Distâncias calculadas em <data>" (dados_mapa.js agora
  carrega um ATUALIZADO gerado junto com os números).
- Páginas de consulta (FAZENDA_X.html) e planilhas recalculadas via o novo
  scripts/publica.py do talhoes-distancias: texto "fechou só com as
  divisas" trocado pelo correto, bancada unificada sem mais desenhar T-40C
  (polígono errado, já excluído do cálculo).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FAZENDA_MATO_GROSSO_distancias.xlsx
+++ b/FAZENDA_MATO_GROSSO_distancias.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\talhao\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\talhoes-distancias\saidas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FB3039B-164B-4D90-AE11-F73633C279E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C338B00E-43F5-4051-A2A4-E00722CD39D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2232" yWindow="2232" windowWidth="14100" windowHeight="9792" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Distâncias" sheetId="1" r:id="rId1"/>

</xml_diff>